<commit_message>
Update docs with 27oct26 changes
</commit_message>
<xml_diff>
--- a/proto_table/elements.xlsx
+++ b/proto_table/elements.xlsx
@@ -20423,7 +20423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20463,6 +20463,966 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>name_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>zinc-ingot</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>zinc</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Zinc ingot</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Lingot de zinc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>zinc-plate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>zinc</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Zinc plate</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Plaque de zinc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>zinc-powder</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>zinc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Zinc powder</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Poudre de zinc</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tin-ingot</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tin</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tin ingot</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Lingot d'étain</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tin-plate</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tin</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tin plate</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Plaque d'étain</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tin-powder</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Tin powder</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Poudre d'étain</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>lead-ingot</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>lead</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Lead ingot</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Lingot de plomb</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>lead-plate</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>lead</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Lead plate</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Plaque de plomb</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lead-powder</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>lead</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Lead powder</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Poudre de plomb</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>nickel-ingot</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>nickel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Nickel ingot</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Lingot de nickel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>nickel-plate</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>nickel</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Nickel plate</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Plaque de nickel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>nickel-powder</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nickel</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Nickel powder</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Poudre de nickel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>aluminium-ingot</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>aluminium</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aluminium ingot</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Lingot d'aluminium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>aluminium-plate</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>aluminium</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Aluminium plate</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Plaque d'aluminium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>aluminium-powder</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>aluminium</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Aluminium powder</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Poudre d'aluminium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>bronze-ingot</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>bronze</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Bronze ingot</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Lingot de bronze</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>bronze-plate</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>bronze</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bronze plate</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Plaque de bronze</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>bronze-powder</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bronze</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Bronze powder</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Poudre de bronze</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>brass-ingot</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>brass</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Brass ingot</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Lingot de laiton</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>brass-plate</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>brass</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Brass plate</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Plaque de laiton</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>brass-powder</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>brass</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>100</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Brass powder</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Poudre de laiton</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>stainless-steel-ingot</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>stainless-steel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Stainless steel ingot</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Lingot d'acier inoxydable</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>stainless-steel-plate</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>stainless-steel</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Stainless steel plate</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Plaque d'acier inoxydable</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>stainless-steel-powder</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>stainless-steel</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Stainless steel powder</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Poudre d'acier inoxydable</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>duralumin-ingot</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>duralumin</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>experimental</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>100</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Duralumin ingot</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Lingot de duralumin</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>duralumin-plate</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>duralumin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>experimental</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Duralumin plate</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Plaque de duralumin</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>duralumin-powder</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>duralumin</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>experimental</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>100</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Duralumin powder</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Poudre de duralumin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>iron-ingot</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Iron ingot</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Lingot de fer</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>iron-powder</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Iron powder</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Poudre de fer</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>copper-ingot</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>100</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Copper ingot</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Lingot de cuivre</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>copper-powder</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Copper powder</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Poudre de cuivre</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>steel-ingot</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Steel ingot</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Lingot d'acier</t>
         </is>
       </c>
     </row>

</xml_diff>